<commit_message>
Cap nhat log va doi ten so do lop
</commit_message>
<xml_diff>
--- a/ai_logs/Tuan_AI_log.xlsx
+++ b/ai_logs/Tuan_AI_log.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="13980"/>
+    <workbookView windowWidth="20745" windowHeight="9480" firstSheet="3" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="1. Metadata &amp; Summary" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="304">
   <si>
     <t>AI Audit Log - Food Delivery System - LAB211</t>
   </si>
@@ -62,7 +62,7 @@
     <t>Assignment:</t>
   </si>
   <si>
-    <t>Food Delivery Network (Mô hình GrabodFo/ShopeeFood)</t>
+    <t>Food Delivery Network (Mô hình GrabFood/ShopeeFood)</t>
   </si>
   <si>
     <t>AI USAGE SUMMARY</t>
@@ -1007,13 +1007,37 @@
     <t>Do I have evidence?</t>
   </si>
   <si>
-    <t>Yes - documented in Human Delta</t>
-  </si>
-  <si>
-    <t>Yes - AI Response column</t>
-  </si>
-  <si>
-    <t>Yes - Evidence column</t>
+    <t>Vì luật môn học cấm Actor trỏ mũi tên kế thừa Actor khác. Làm phẳng sơ đồ giúp dễ bóc tách logic hơn.</t>
+  </si>
+  <si>
+    <t>Nhớ rõ. AI từng xúi gộp chung đăng nhập vào 1 Actor cha tên là 'User'</t>
+  </si>
+  <si>
+    <t>Có. Sơ đồ Use Case cuối cùng trong file report.docx.</t>
+  </si>
+  <si>
+    <t>05</t>
+  </si>
+  <si>
+    <t>Cần công thức tính khoảng cách GPS. Tự code cứng bán kính Trái Đất R = 6371km để tối ưu.</t>
+  </si>
+  <si>
+    <t>AI cho code đúng nhưng lại 'bịa' ra việc công thức này thuộc chuẩn IEEE 2024 Geo-routing.</t>
+  </si>
+  <si>
+    <t>File GeoUtils.java và log ChatGPT.</t>
+  </si>
+  <si>
+    <t>09</t>
+  </si>
+  <si>
+    <t>Dùng Hashmap để Lock theo từng ID món ăn, thay vì Lock toàn bộ hàm. Giúp giữ Throughput không bị giảm quá 30%</t>
+  </si>
+  <si>
+    <t>AI khuyên dùng từ khóa synchronized cứng cho cả hàm deductStock() -&gt; dẫn đến thắt cổ chai.</t>
+  </si>
+  <si>
+    <t>Mở file CsvRepository.java, chỉ cho thầy xem dòng code hàm deductStock.</t>
   </si>
 </sst>
 </file>
@@ -1027,7 +1051,7 @@
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="178" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="33">
+  <fonts count="34">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1101,6 +1125,11 @@
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8.8"/>
+      <name val="Consolas"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
@@ -1629,137 +1658,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1789,18 +1818,21 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1808,11 +1840,14 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2162,16 +2197,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F28"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.3" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
-    <col min="3" max="3" width="52.716814159292" customWidth="1"/>
+    <col min="3" max="3" width="52.7142857142857" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
     <col min="5" max="6" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20.65" spans="1:5">
+    <row r="1" ht="21" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2181,13 +2216,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" ht="18" spans="1:5">
+    <row r="3" ht="18.75" spans="1:5">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="20" t="s">
         <v>3</v>
       </c>
       <c r="C4" t="s">
@@ -2195,7 +2230,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="20" t="s">
         <v>5</v>
       </c>
       <c r="C5" t="s">
@@ -2203,7 +2238,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="20" t="s">
         <v>7</v>
       </c>
       <c r="C6" t="s">
@@ -2211,20 +2246,20 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="C7" s="21" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="9" ht="18" spans="1:5">
+    <row r="9" ht="18.75" spans="1:5">
       <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="20" t="s">
         <v>12</v>
       </c>
       <c r="C10" t="s">
@@ -2232,38 +2267,38 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="21">
+      <c r="C11" s="22">
         <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="22">
+      <c r="C12" s="23">
         <v>0.16</v>
       </c>
-      <c r="E12" s="23" t="s">
+      <c r="E12" s="24" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="21">
+      <c r="C13" s="22">
         <v>6</v>
       </c>
     </row>
-    <row r="15" ht="18" spans="1:5">
+    <row r="15" ht="18.75" spans="1:5">
       <c r="A15" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="16" ht="14.35" spans="1:5">
+    <row r="16" spans="1:5">
       <c r="A16" s="4" t="s">
         <v>19</v>
       </c>
@@ -2277,7 +2312,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" ht="14.35" spans="1:4">
+    <row r="17" spans="1:4">
       <c r="A17" s="14" t="s">
         <v>23</v>
       </c>
@@ -2291,7 +2326,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="18" ht="14.35" spans="1:4">
+    <row r="18" spans="1:4">
       <c r="A18" s="14" t="s">
         <v>27</v>
       </c>
@@ -2305,7 +2340,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="19" ht="14.35" spans="1:4">
+    <row r="19" ht="30" spans="1:4">
       <c r="A19" s="14" t="s">
         <v>31</v>
       </c>
@@ -2319,7 +2354,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="20" ht="14.35" spans="1:4">
+    <row r="20" spans="1:4">
       <c r="A20" s="14"/>
       <c r="B20" s="14"/>
       <c r="C20" s="14"/>
@@ -2327,12 +2362,12 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" ht="18" spans="1:4">
+    <row r="22" ht="18.75" spans="1:4">
       <c r="A22" s="3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="23" ht="14.35" spans="1:4">
+    <row r="23" spans="1:4">
       <c r="A23" s="4" t="s">
         <v>37</v>
       </c>
@@ -2343,47 +2378,47 @@
         <v>39</v>
       </c>
     </row>
-    <row r="24" ht="14.35" spans="1:4">
+    <row r="24" spans="1:4">
       <c r="A24" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="B24" s="24">
+      <c r="B24" s="25">
         <v>4</v>
       </c>
-      <c r="C24" s="13" t="s">
+      <c r="C24" s="15" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="25" ht="14.35" spans="1:4">
+    <row r="25" spans="1:4">
       <c r="A25" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="B25" s="24">
+      <c r="B25" s="25">
         <v>10</v>
       </c>
-      <c r="C25" s="13" t="s">
+      <c r="C25" s="15" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="26" ht="14.35" spans="1:4">
+    <row r="26" spans="1:4">
       <c r="A26" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="B26" s="24">
+      <c r="B26" s="25">
         <v>5</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="C26" s="15" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="27" ht="14.35" spans="1:4">
+    <row r="27" spans="1:4">
       <c r="A27" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="B27" s="24">
+      <c r="B27" s="25">
         <v>8</v>
       </c>
-      <c r="C27" s="13" t="s">
+      <c r="C27" s="15" t="s">
         <v>41</v>
       </c>
     </row>
@@ -2408,7 +2443,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:H35"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.3" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="3" width="18" customWidth="1"/>
@@ -2419,13 +2454,13 @@
     <col min="8" max="8" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20.65" spans="1:8">
+    <row r="1" ht="21" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:8">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>47</v>
       </c>
     </row>
@@ -3053,7 +3088,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="27" ht="114.65" spans="1:8">
+    <row r="27" ht="120" spans="1:8">
       <c r="A27">
         <v>24</v>
       </c>
@@ -3072,14 +3107,14 @@
       <c r="F27" t="s">
         <v>164</v>
       </c>
-      <c r="G27" s="18" t="s">
+      <c r="G27" s="19" t="s">
         <v>165</v>
       </c>
       <c r="H27" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="28" ht="114.65" spans="1:8">
+    <row r="28" ht="120" spans="1:8">
       <c r="A28">
         <v>25</v>
       </c>
@@ -3098,14 +3133,14 @@
       <c r="F28" t="s">
         <v>169</v>
       </c>
-      <c r="G28" s="18" t="s">
+      <c r="G28" s="19" t="s">
         <v>170</v>
       </c>
       <c r="H28" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="29" ht="114.65" spans="1:8">
+    <row r="29" ht="120" spans="1:8">
       <c r="A29">
         <v>26</v>
       </c>
@@ -3124,14 +3159,14 @@
       <c r="F29" t="s">
         <v>173</v>
       </c>
-      <c r="G29" s="18" t="s">
+      <c r="G29" s="19" t="s">
         <v>174</v>
       </c>
       <c r="H29" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="30" ht="100.35" spans="1:8">
+    <row r="30" ht="120" spans="1:8">
       <c r="A30">
         <v>27</v>
       </c>
@@ -3150,14 +3185,14 @@
       <c r="F30" t="s">
         <v>178</v>
       </c>
-      <c r="G30" s="18" t="s">
+      <c r="G30" s="19" t="s">
         <v>179</v>
       </c>
       <c r="H30" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="31" ht="114.65" spans="1:8">
+    <row r="31" ht="120" spans="1:8">
       <c r="A31">
         <v>28</v>
       </c>
@@ -3176,14 +3211,14 @@
       <c r="F31" t="s">
         <v>182</v>
       </c>
-      <c r="G31" s="18" t="s">
+      <c r="G31" s="19" t="s">
         <v>183</v>
       </c>
       <c r="H31" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="32" ht="100.35" spans="1:8">
+    <row r="32" ht="135" spans="1:8">
       <c r="A32">
         <v>29</v>
       </c>
@@ -3202,14 +3237,14 @@
       <c r="F32" t="s">
         <v>187</v>
       </c>
-      <c r="G32" s="18" t="s">
+      <c r="G32" s="19" t="s">
         <v>188</v>
       </c>
       <c r="H32" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="33" ht="114.65" spans="1:8">
+    <row r="33" ht="120" spans="1:8">
       <c r="A33">
         <v>30</v>
       </c>
@@ -3228,14 +3263,14 @@
       <c r="F33" t="s">
         <v>192</v>
       </c>
-      <c r="G33" s="18" t="s">
+      <c r="G33" s="19" t="s">
         <v>193</v>
       </c>
       <c r="H33" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="34" ht="100.35" spans="1:8">
+    <row r="34" ht="120" spans="1:8">
       <c r="A34">
         <v>31</v>
       </c>
@@ -3254,14 +3289,14 @@
       <c r="F34" t="s">
         <v>196</v>
       </c>
-      <c r="G34" s="18" t="s">
+      <c r="G34" s="19" t="s">
         <v>197</v>
       </c>
       <c r="H34" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="35" ht="114.65" spans="1:8">
+    <row r="35" ht="120" spans="1:8">
       <c r="A35">
         <v>32</v>
       </c>
@@ -3280,7 +3315,7 @@
       <c r="F35" t="s">
         <v>200</v>
       </c>
-      <c r="G35" s="18" t="s">
+      <c r="G35" s="19" t="s">
         <v>201</v>
       </c>
       <c r="H35" t="s">
@@ -3301,20 +3336,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F36"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.3" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
     <col min="3" max="6" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20.65" spans="1:6">
-      <c r="A1" s="15" t="s">
+    <row r="1" ht="21" spans="1:6">
+      <c r="A1" s="16" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="17" t="s">
         <v>203</v>
       </c>
     </row>
@@ -3358,7 +3393,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="5" ht="57.35" spans="1:6">
+    <row r="5" ht="60" spans="1:6">
       <c r="A5" s="14">
         <v>16</v>
       </c>
@@ -3578,12 +3613,12 @@
       <c r="E24" s="14"/>
       <c r="F24" s="14"/>
     </row>
-    <row r="30" ht="18" spans="1:6">
+    <row r="30" ht="18.75" spans="1:6">
       <c r="A30" s="3" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="31" ht="14.35" spans="1:6">
+    <row r="31" spans="1:6">
       <c r="A31" s="12" t="s">
         <v>239</v>
       </c>
@@ -3594,7 +3629,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="32" ht="28.65" spans="1:6">
+    <row r="32" ht="30" spans="1:6">
       <c r="A32" s="14" t="s">
         <v>218</v>
       </c>
@@ -3605,7 +3640,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="33" ht="28.65" spans="1:3">
+    <row r="33" ht="30" spans="1:3">
       <c r="A33" s="14" t="s">
         <v>244</v>
       </c>
@@ -3616,7 +3651,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="34" ht="28.65" spans="1:3">
+    <row r="34" ht="30" spans="1:3">
       <c r="A34" s="14" t="s">
         <v>247</v>
       </c>
@@ -3627,7 +3662,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="35" ht="28.65" spans="1:3">
+    <row r="35" ht="30" spans="1:3">
       <c r="A35" s="14" t="s">
         <v>250</v>
       </c>
@@ -3638,7 +3673,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="36" ht="43" spans="1:3">
+    <row r="36" ht="45" spans="1:3">
       <c r="A36" s="14" t="s">
         <v>209</v>
       </c>
@@ -3662,16 +3697,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D33"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.3" outlineLevelCol="3"/>
+  <dimension ref="A1:D30"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="3" max="3" width="25.7142857142857" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20.65" spans="1:4">
+    <row r="1" ht="21" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>255</v>
       </c>
@@ -3681,12 +3716,12 @@
         <v>256</v>
       </c>
     </row>
-    <row r="4" ht="18" spans="1:4">
+    <row r="4" ht="18.75" spans="1:4">
       <c r="A4" s="3" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="5" ht="14.35" spans="1:4">
+    <row r="5" spans="1:4">
       <c r="A5" s="4" t="s">
         <v>258</v>
       </c>
@@ -3700,7 +3735,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="6" ht="26" spans="1:4">
+    <row r="6" ht="25.5" spans="1:4">
       <c r="A6" s="6">
         <v>1</v>
       </c>
@@ -3714,7 +3749,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="7" ht="26" spans="1:4">
+    <row r="7" ht="25.5" spans="1:4">
       <c r="A7" s="6">
         <v>2</v>
       </c>
@@ -3728,7 +3763,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="8" ht="26" spans="1:4">
+    <row r="8" ht="25.5" spans="1:4">
       <c r="A8" s="6">
         <v>3</v>
       </c>
@@ -3742,7 +3777,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="9" ht="26" spans="1:4">
+    <row r="9" ht="25.5" spans="1:4">
       <c r="A9" s="6">
         <v>4</v>
       </c>
@@ -3756,7 +3791,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="10" ht="26" spans="1:4">
+    <row r="10" ht="25.5" spans="1:4">
       <c r="A10" s="6">
         <v>5</v>
       </c>
@@ -3770,12 +3805,12 @@
         <v>272</v>
       </c>
     </row>
-    <row r="12" ht="18" spans="1:4">
+    <row r="12" ht="18.75" spans="1:4">
       <c r="A12" s="3" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="13" ht="14.35" spans="1:4">
+    <row r="13" spans="1:4">
       <c r="A13" s="4" t="s">
         <v>258</v>
       </c>
@@ -3803,7 +3838,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="15" ht="26" spans="1:4">
+    <row r="15" ht="25.5" spans="1:4">
       <c r="A15" s="6">
         <v>2</v>
       </c>
@@ -3845,7 +3880,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="18" ht="26" spans="1:4">
+    <row r="18" ht="25.5" spans="1:4">
       <c r="A18" s="6">
         <v>5</v>
       </c>
@@ -3859,7 +3894,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="20" ht="15.65" spans="1:4">
+    <row r="20" ht="15.75" spans="1:4">
       <c r="A20" s="8" t="s">
         <v>285</v>
       </c>
@@ -3874,7 +3909,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="25" ht="18" spans="1:4">
+    <row r="25" ht="18.75" spans="1:4">
       <c r="A25" s="3" t="s">
         <v>288</v>
       </c>
@@ -3884,7 +3919,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="27" ht="57.35" spans="1:4">
+    <row r="27" ht="30" spans="1:4">
       <c r="A27" s="11" t="s">
         <v>48</v>
       </c>
@@ -3898,9 +3933,9 @@
         <v>292</v>
       </c>
     </row>
-    <row r="28" ht="43" spans="1:4">
+    <row r="28" ht="50" customHeight="1" spans="1:4">
       <c r="A28" s="13">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="B28" s="14" t="s">
         <v>293</v>
@@ -3912,74 +3947,32 @@
         <v>295</v>
       </c>
     </row>
-    <row r="29" ht="43" spans="1:4">
-      <c r="A29" s="13">
-        <v>8</v>
+    <row r="29" ht="60" spans="1:4">
+      <c r="A29" s="26" t="s">
+        <v>296</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="30" ht="43" spans="1:4">
-      <c r="A30" s="13">
-        <v>12</v>
+        <v>299</v>
+      </c>
+    </row>
+    <row r="30" ht="60" spans="1:4">
+      <c r="A30" s="26" t="s">
+        <v>300</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4">
-      <c r="A31">
-        <v>16</v>
-      </c>
-      <c r="B31" t="s">
-        <v>293</v>
-      </c>
-      <c r="C31" t="s">
-        <v>294</v>
-      </c>
-      <c r="D31" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4">
-      <c r="A32">
-        <v>25</v>
-      </c>
-      <c r="B32" t="s">
-        <v>293</v>
-      </c>
-      <c r="C32" t="s">
-        <v>294</v>
-      </c>
-      <c r="D32" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4">
-      <c r="A33">
-        <v>26</v>
-      </c>
-      <c r="B33" t="s">
-        <v>293</v>
-      </c>
-      <c r="C33" t="s">
-        <v>294</v>
-      </c>
-      <c r="D33" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
     </row>
   </sheetData>

</xml_diff>